<commit_message>
Milestone 8A UK Peppol readiness XML
</commit_message>
<xml_diff>
--- a/test_data/workbooks/UK-PEPPOL-SANDBOX-001.xlsx
+++ b/test_data/workbooks/UK-PEPPOL-SANDBOX-001.xlsx
@@ -534,12 +534,12 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>0088:123456789</t>
+          <t>9932:GB123456789</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0088</t>
+          <t>9932</t>
         </is>
       </c>
     </row>
@@ -682,12 +682,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0088:987654321</t>
+          <t>9932:GB987654321</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>0088</t>
+          <t>9932</t>
         </is>
       </c>
     </row>
@@ -875,7 +875,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>storecove_peppol_sandbox_readiness_test</t>
+          <t>uk_peppol_readiness_ubl</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>UK Peppol sandbox readiness sample.</t>
+          <t>UK Peppol readiness XML sample.</t>
         </is>
       </c>
     </row>

</xml_diff>